<commit_message>
Daily recap, matchup updates, learning and research 2026-08-29
</commit_message>
<xml_diff>
--- a/data/k-props/2026-08-29.xlsx
+++ b/data/k-props/2026-08-29.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="101">
   <si>
     <t>date</t>
   </si>
@@ -145,21 +145,30 @@
     <t>lineup_unweighted_30d_posted</t>
   </si>
   <si>
+    <t>O</t>
+  </si>
+  <si>
+    <t>W</t>
+  </si>
+  <si>
+    <t>&lt;6</t>
+  </si>
+  <si>
+    <t>Carlos Rodón</t>
+  </si>
+  <si>
+    <t>U</t>
+  </si>
+  <si>
+    <t>Alec Gamboa</t>
+  </si>
+  <si>
+    <t>Opener / bullpen game</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
-    <t>&lt;6</t>
-  </si>
-  <si>
-    <t>Carlos Rodón</t>
-  </si>
-  <si>
-    <t>Alec Gamboa</t>
-  </si>
-  <si>
-    <t>Opener / bullpen game</t>
-  </si>
-  <si>
     <t>Max Fried</t>
   </si>
   <si>
@@ -230,6 +239,9 @@
   </si>
   <si>
     <t>Cade Cavalli</t>
+  </si>
+  <si>
+    <t>L</t>
   </si>
   <si>
     <t>Daniel Lynch IV</t>
@@ -883,17 +895,23 @@
       <c r="Y2">
         <v>1.0351</v>
       </c>
+      <c r="Z2">
+        <v>7</v>
+      </c>
       <c r="AA2" t="s">
         <v>44</v>
       </c>
+      <c r="AB2">
+        <v>1.62</v>
+      </c>
       <c r="AC2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD2">
         <v>5.9</v>
       </c>
       <c r="AE2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF2">
         <v>0.2135</v>
@@ -903,6 +921,18 @@
       </c>
       <c r="AH2">
         <v>0.22</v>
+      </c>
+      <c r="AI2">
+        <v>1.1</v>
+      </c>
+      <c r="AJ2">
+        <v>1.1</v>
+      </c>
+      <c r="AK2">
+        <v>0.88</v>
+      </c>
+      <c r="AL2">
+        <v>0.88</v>
       </c>
       <c r="AM2">
         <v>6.12</v>
@@ -913,7 +943,7 @@
         <v>39</v>
       </c>
       <c r="B3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C3">
         <v>5.5</v>
@@ -984,17 +1014,23 @@
       <c r="Y3">
         <v>0.9697</v>
       </c>
+      <c r="Z3">
+        <v>5</v>
+      </c>
       <c r="AA3" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB3">
+        <v>-1.01</v>
       </c>
       <c r="AC3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD3">
         <v>4.27</v>
       </c>
       <c r="AE3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF3">
         <v>0.2467</v>
@@ -1004,6 +1040,18 @@
       </c>
       <c r="AH3">
         <v>0.22</v>
+      </c>
+      <c r="AI3">
+        <v>0.73</v>
+      </c>
+      <c r="AJ3">
+        <v>0.73</v>
+      </c>
+      <c r="AK3">
+        <v>0.51</v>
+      </c>
+      <c r="AL3">
+        <v>0.51</v>
       </c>
       <c r="AM3">
         <v>4.49</v>
@@ -1014,7 +1062,7 @@
         <v>39</v>
       </c>
       <c r="B4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="F4" t="s">
         <v>41</v>
@@ -1023,7 +1071,7 @@
         <v>823501</v>
       </c>
       <c r="H4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="I4">
         <v>1.3</v>
@@ -1077,16 +1125,16 @@
         <v>1.0597</v>
       </c>
       <c r="AA4" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="AC4" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="AD4">
         <v>1.19</v>
       </c>
       <c r="AE4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF4">
         <v>0.1784</v>
@@ -1106,7 +1154,7 @@
         <v>39</v>
       </c>
       <c r="B5" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="C5">
         <v>4.5</v>
@@ -1177,17 +1225,23 @@
       <c r="Y5">
         <v>0.9794</v>
       </c>
+      <c r="Z5">
+        <v>4</v>
+      </c>
       <c r="AA5" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB5">
+        <v>0.26</v>
       </c>
       <c r="AC5" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="AD5">
         <v>4.54</v>
       </c>
       <c r="AE5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF5">
         <v>0.2537</v>
@@ -1197,6 +1251,18 @@
       </c>
       <c r="AH5">
         <v>0.22</v>
+      </c>
+      <c r="AI5">
+        <v>-0.54</v>
+      </c>
+      <c r="AJ5">
+        <v>0.54</v>
+      </c>
+      <c r="AK5">
+        <v>-0.76</v>
+      </c>
+      <c r="AL5">
+        <v>0.76</v>
       </c>
       <c r="AM5">
         <v>4.76</v>
@@ -1207,7 +1273,7 @@
         <v>39</v>
       </c>
       <c r="B6" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C6">
         <v>6.5</v>
@@ -1219,7 +1285,7 @@
         <v>-105</v>
       </c>
       <c r="F6" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="G6">
         <v>824230</v>
@@ -1278,17 +1344,23 @@
       <c r="Y6">
         <v>0.9742</v>
       </c>
+      <c r="Z6">
+        <v>10</v>
+      </c>
       <c r="AA6" t="s">
         <v>44</v>
       </c>
+      <c r="AB6">
+        <v>-0.12</v>
+      </c>
       <c r="AC6" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="AD6">
         <v>6.93</v>
       </c>
       <c r="AE6" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="AF6">
         <v>0.3303</v>
@@ -1298,6 +1370,18 @@
       </c>
       <c r="AH6">
         <v>-0.55</v>
+      </c>
+      <c r="AI6">
+        <v>3.07</v>
+      </c>
+      <c r="AJ6">
+        <v>3.07</v>
+      </c>
+      <c r="AK6">
+        <v>3.62</v>
+      </c>
+      <c r="AL6">
+        <v>3.62</v>
       </c>
       <c r="AM6">
         <v>6.38</v>
@@ -1308,7 +1392,7 @@
         <v>39</v>
       </c>
       <c r="B7" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C7">
         <v>3.5</v>
@@ -1320,7 +1404,7 @@
         <v>-115</v>
       </c>
       <c r="F7" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="G7">
         <v>824230</v>
@@ -1379,17 +1463,23 @@
       <c r="Y7">
         <v>0.991</v>
       </c>
+      <c r="Z7">
+        <v>3</v>
+      </c>
       <c r="AA7" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB7">
+        <v>-0.09</v>
       </c>
       <c r="AC7" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="AD7">
         <v>3.19</v>
       </c>
       <c r="AE7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF7">
         <v>0.1473</v>
@@ -1399,6 +1489,18 @@
       </c>
       <c r="AH7">
         <v>0.22</v>
+      </c>
+      <c r="AI7">
+        <v>-0.19</v>
+      </c>
+      <c r="AJ7">
+        <v>0.19</v>
+      </c>
+      <c r="AK7">
+        <v>-0.41</v>
+      </c>
+      <c r="AL7">
+        <v>0.41</v>
       </c>
       <c r="AM7">
         <v>3.41</v>
@@ -1409,10 +1511,10 @@
         <v>39</v>
       </c>
       <c r="B8" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="F8" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G8">
         <v>823665</v>
@@ -1472,16 +1574,16 @@
         <v>0.936</v>
       </c>
       <c r="AA8" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="AC8" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="AD8">
         <v>3.27</v>
       </c>
       <c r="AE8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF8">
         <v>0.1833</v>
@@ -1501,10 +1603,10 @@
         <v>39</v>
       </c>
       <c r="B9" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="F9" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G9">
         <v>823665</v>
@@ -1564,16 +1666,16 @@
         <v>1.0323</v>
       </c>
       <c r="AA9" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="AC9" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="AD9">
         <v>4.23</v>
       </c>
       <c r="AE9" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF9">
         <v>0.158</v>
@@ -1593,16 +1695,16 @@
         <v>39</v>
       </c>
       <c r="B10" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="F10" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="G10">
         <v>823011</v>
       </c>
       <c r="H10" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="I10">
         <v>2.3</v>
@@ -1656,16 +1758,16 @@
         <v>0.8961</v>
       </c>
       <c r="AA10" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="AC10" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="AD10">
         <v>2.45</v>
       </c>
       <c r="AE10" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF10">
         <v>0.252</v>
@@ -1685,10 +1787,10 @@
         <v>39</v>
       </c>
       <c r="B11" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="F11" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="G11">
         <v>823011</v>
@@ -1748,16 +1850,16 @@
         <v>1.0293</v>
       </c>
       <c r="AA11" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="AC11" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="AD11">
         <v>5.97</v>
       </c>
       <c r="AE11" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF11">
         <v>0.2433</v>
@@ -1777,7 +1879,7 @@
         <v>39</v>
       </c>
       <c r="B12" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C12">
         <v>3.5</v>
@@ -1789,7 +1891,7 @@
         <v>126</v>
       </c>
       <c r="F12" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="G12">
         <v>824637</v>
@@ -1848,17 +1950,23 @@
       <c r="Y12">
         <v>0.8905</v>
       </c>
+      <c r="Z12">
+        <v>1</v>
+      </c>
       <c r="AA12" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB12">
+        <v>-0.59</v>
       </c>
       <c r="AC12" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="AD12">
         <v>2.69</v>
       </c>
       <c r="AE12" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF12">
         <v>0.1727</v>
@@ -1868,6 +1976,18 @@
       </c>
       <c r="AH12">
         <v>0.22</v>
+      </c>
+      <c r="AI12">
+        <v>-1.69</v>
+      </c>
+      <c r="AJ12">
+        <v>1.69</v>
+      </c>
+      <c r="AK12">
+        <v>-1.91</v>
+      </c>
+      <c r="AL12">
+        <v>1.91</v>
       </c>
       <c r="AM12">
         <v>2.91</v>
@@ -1878,7 +1998,7 @@
         <v>39</v>
       </c>
       <c r="B13" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C13">
         <v>6.5</v>
@@ -1890,7 +2010,7 @@
         <v>-130</v>
       </c>
       <c r="F13" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="G13">
         <v>824637</v>
@@ -1949,17 +2069,23 @@
       <c r="Y13">
         <v>1.12</v>
       </c>
+      <c r="Z13">
+        <v>7</v>
+      </c>
       <c r="AA13" t="s">
         <v>44</v>
       </c>
+      <c r="AB13">
+        <v>0.87</v>
+      </c>
       <c r="AC13" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD13">
         <v>7.37</v>
       </c>
       <c r="AE13" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="AF13">
         <v>0.2423</v>
@@ -1969,6 +2095,18 @@
       </c>
       <c r="AH13">
         <v>0</v>
+      </c>
+      <c r="AI13">
+        <v>-0.37</v>
+      </c>
+      <c r="AJ13">
+        <v>0.37</v>
+      </c>
+      <c r="AK13">
+        <v>-0.37</v>
+      </c>
+      <c r="AL13">
+        <v>0.37</v>
       </c>
       <c r="AM13">
         <v>7.37</v>
@@ -1979,7 +2117,7 @@
         <v>39</v>
       </c>
       <c r="B14" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="C14">
         <v>5.5</v>
@@ -1991,7 +2129,7 @@
         <v>-130</v>
       </c>
       <c r="F14" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="G14">
         <v>822770</v>
@@ -2050,17 +2188,23 @@
       <c r="Y14">
         <v>0.9726</v>
       </c>
+      <c r="Z14">
+        <v>6</v>
+      </c>
       <c r="AA14" t="s">
         <v>44</v>
       </c>
+      <c r="AB14">
+        <v>0.7</v>
+      </c>
       <c r="AC14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD14">
         <v>5.98</v>
       </c>
       <c r="AE14" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF14">
         <v>0.2172</v>
@@ -2070,6 +2214,18 @@
       </c>
       <c r="AH14">
         <v>0.22</v>
+      </c>
+      <c r="AI14">
+        <v>0.02</v>
+      </c>
+      <c r="AJ14">
+        <v>0.02</v>
+      </c>
+      <c r="AK14">
+        <v>-0.2</v>
+      </c>
+      <c r="AL14">
+        <v>0.2</v>
       </c>
       <c r="AM14">
         <v>6.2</v>
@@ -2080,7 +2236,7 @@
         <v>39</v>
       </c>
       <c r="B15" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C15">
         <v>4.5</v>
@@ -2092,7 +2248,7 @@
         <v>-170</v>
       </c>
       <c r="F15" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="G15">
         <v>823177</v>
@@ -2151,17 +2307,23 @@
       <c r="Y15">
         <v>0.9313</v>
       </c>
+      <c r="Z15">
+        <v>7</v>
+      </c>
       <c r="AA15" t="s">
         <v>44</v>
       </c>
+      <c r="AB15">
+        <v>-0.48</v>
+      </c>
       <c r="AC15" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="AD15">
         <v>3.8</v>
       </c>
       <c r="AE15" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF15">
         <v>0.1567</v>
@@ -2171,6 +2333,18 @@
       </c>
       <c r="AH15">
         <v>0.22</v>
+      </c>
+      <c r="AI15">
+        <v>3.2</v>
+      </c>
+      <c r="AJ15">
+        <v>3.2</v>
+      </c>
+      <c r="AK15">
+        <v>2.98</v>
+      </c>
+      <c r="AL15">
+        <v>2.98</v>
       </c>
       <c r="AM15">
         <v>4.02</v>
@@ -2181,7 +2355,7 @@
         <v>39</v>
       </c>
       <c r="B16" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="C16">
         <v>3.5</v>
@@ -2193,13 +2367,13 @@
         <v>-104</v>
       </c>
       <c r="F16" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="G16">
         <v>823176</v>
       </c>
       <c r="H16" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="I16">
         <v>4.4</v>
@@ -2252,17 +2426,23 @@
       <c r="Y16">
         <v>1.0677</v>
       </c>
+      <c r="Z16">
+        <v>2</v>
+      </c>
       <c r="AA16" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB16">
+        <v>0.66</v>
       </c>
       <c r="AC16" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="AD16">
         <v>3.94</v>
       </c>
       <c r="AE16" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF16">
         <v>0.1666</v>
@@ -2272,6 +2452,18 @@
       </c>
       <c r="AH16">
         <v>0.22</v>
+      </c>
+      <c r="AI16">
+        <v>-1.94</v>
+      </c>
+      <c r="AJ16">
+        <v>1.94</v>
+      </c>
+      <c r="AK16">
+        <v>-2.16</v>
+      </c>
+      <c r="AL16">
+        <v>2.16</v>
       </c>
       <c r="AM16">
         <v>4.16</v>
@@ -2282,7 +2474,7 @@
         <v>39</v>
       </c>
       <c r="B17" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="C17">
         <v>4.5</v>
@@ -2294,7 +2486,7 @@
         <v>-150</v>
       </c>
       <c r="F17" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="G17">
         <v>822690</v>
@@ -2353,17 +2545,23 @@
       <c r="Y17">
         <v>0.9921</v>
       </c>
+      <c r="Z17">
+        <v>3</v>
+      </c>
       <c r="AA17" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB17">
+        <v>0.4</v>
       </c>
       <c r="AC17" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="AD17">
         <v>4.68</v>
       </c>
       <c r="AE17" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF17">
         <v>0.1663</v>
@@ -2373,6 +2571,18 @@
       </c>
       <c r="AH17">
         <v>0.22</v>
+      </c>
+      <c r="AI17">
+        <v>-1.68</v>
+      </c>
+      <c r="AJ17">
+        <v>1.68</v>
+      </c>
+      <c r="AK17">
+        <v>-1.9</v>
+      </c>
+      <c r="AL17">
+        <v>1.9</v>
       </c>
       <c r="AM17">
         <v>4.9</v>
@@ -2383,7 +2593,7 @@
         <v>39</v>
       </c>
       <c r="B18" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C18">
         <v>6.5</v>
@@ -2395,7 +2605,7 @@
         <v>-128</v>
       </c>
       <c r="F18" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="G18">
         <v>822690</v>
@@ -2454,17 +2664,23 @@
       <c r="Y18">
         <v>0.9439</v>
       </c>
+      <c r="Z18">
+        <v>8</v>
+      </c>
       <c r="AA18" t="s">
         <v>44</v>
       </c>
+      <c r="AB18">
+        <v>-0.82</v>
+      </c>
       <c r="AC18" t="s">
-        <v>44</v>
+        <v>76</v>
       </c>
       <c r="AD18">
         <v>6.23</v>
       </c>
       <c r="AE18" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="AF18">
         <v>0.3163</v>
@@ -2474,6 +2690,18 @@
       </c>
       <c r="AH18">
         <v>-0.55</v>
+      </c>
+      <c r="AI18">
+        <v>1.77</v>
+      </c>
+      <c r="AJ18">
+        <v>1.77</v>
+      </c>
+      <c r="AK18">
+        <v>2.32</v>
+      </c>
+      <c r="AL18">
+        <v>2.32</v>
       </c>
       <c r="AM18">
         <v>5.68</v>
@@ -2484,7 +2712,7 @@
         <v>39</v>
       </c>
       <c r="B19" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="C19">
         <v>2.5</v>
@@ -2496,13 +2724,13 @@
         <v>-107</v>
       </c>
       <c r="F19" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="G19">
         <v>824392</v>
       </c>
       <c r="H19" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="I19">
         <v>3</v>
@@ -2555,17 +2783,23 @@
       <c r="Y19">
         <v>0.88</v>
       </c>
+      <c r="Z19">
+        <v>3</v>
+      </c>
       <c r="AA19" t="s">
         <v>44</v>
       </c>
+      <c r="AB19">
+        <v>-0.55</v>
+      </c>
       <c r="AC19" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="AD19">
         <v>1.73</v>
       </c>
       <c r="AE19" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF19">
         <v>0.179</v>
@@ -2575,6 +2809,18 @@
       </c>
       <c r="AH19">
         <v>0.22</v>
+      </c>
+      <c r="AI19">
+        <v>1.27</v>
+      </c>
+      <c r="AJ19">
+        <v>1.27</v>
+      </c>
+      <c r="AK19">
+        <v>1.05</v>
+      </c>
+      <c r="AL19">
+        <v>1.05</v>
       </c>
       <c r="AM19">
         <v>1.95</v>
@@ -2585,7 +2831,7 @@
         <v>39</v>
       </c>
       <c r="B20" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C20">
         <v>5.5</v>
@@ -2597,7 +2843,7 @@
         <v>-108</v>
       </c>
       <c r="F20" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="G20">
         <v>824392</v>
@@ -2656,17 +2902,23 @@
       <c r="Y20">
         <v>1.0087</v>
       </c>
+      <c r="Z20">
+        <v>4</v>
+      </c>
       <c r="AA20" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB20">
+        <v>-0.4</v>
       </c>
       <c r="AC20" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="AD20">
         <v>4.88</v>
       </c>
       <c r="AE20" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF20">
         <v>0.2194</v>
@@ -2676,6 +2928,18 @@
       </c>
       <c r="AH20">
         <v>0.22</v>
+      </c>
+      <c r="AI20">
+        <v>-0.88</v>
+      </c>
+      <c r="AJ20">
+        <v>0.88</v>
+      </c>
+      <c r="AK20">
+        <v>-1.1</v>
+      </c>
+      <c r="AL20">
+        <v>1.1</v>
       </c>
       <c r="AM20">
         <v>5.1</v>
@@ -2686,16 +2950,16 @@
         <v>39</v>
       </c>
       <c r="B21" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F21" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="G21">
         <v>823582</v>
       </c>
       <c r="H21" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="I21">
         <v>1</v>
@@ -2749,16 +3013,16 @@
         <v>0.9768</v>
       </c>
       <c r="AA21" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="AC21" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="AD21">
         <v>1.14</v>
       </c>
       <c r="AE21" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF21">
         <v>0.2203</v>
@@ -2778,7 +3042,7 @@
         <v>39</v>
       </c>
       <c r="B22" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="C22">
         <v>5.5</v>
@@ -2790,7 +3054,7 @@
         <v>116</v>
       </c>
       <c r="F22" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="G22">
         <v>823582</v>
@@ -2849,17 +3113,23 @@
       <c r="Y22">
         <v>0.9509</v>
       </c>
+      <c r="Z22">
+        <v>4</v>
+      </c>
       <c r="AA22" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB22">
+        <v>-0.2</v>
       </c>
       <c r="AC22" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="AD22">
         <v>5.08</v>
       </c>
       <c r="AE22" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF22">
         <v>0.2404</v>
@@ -2869,6 +3139,18 @@
       </c>
       <c r="AH22">
         <v>0.22</v>
+      </c>
+      <c r="AI22">
+        <v>-1.08</v>
+      </c>
+      <c r="AJ22">
+        <v>1.08</v>
+      </c>
+      <c r="AK22">
+        <v>-1.3</v>
+      </c>
+      <c r="AL22">
+        <v>1.3</v>
       </c>
       <c r="AM22">
         <v>5.3</v>
@@ -2879,7 +3161,7 @@
         <v>39</v>
       </c>
       <c r="B23" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="C23">
         <v>3.5</v>
@@ -2891,7 +3173,7 @@
         <v>-122</v>
       </c>
       <c r="F23" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="G23">
         <v>822936</v>
@@ -2950,17 +3232,23 @@
       <c r="Y23">
         <v>0.88</v>
       </c>
+      <c r="Z23">
+        <v>3</v>
+      </c>
       <c r="AA23" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB23">
+        <v>-0.85</v>
       </c>
       <c r="AC23" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD23">
         <v>2.43</v>
       </c>
       <c r="AE23" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF23">
         <v>0.1931</v>
@@ -2970,6 +3258,18 @@
       </c>
       <c r="AH23">
         <v>0.22</v>
+      </c>
+      <c r="AI23">
+        <v>0.57</v>
+      </c>
+      <c r="AJ23">
+        <v>0.57</v>
+      </c>
+      <c r="AK23">
+        <v>0.35</v>
+      </c>
+      <c r="AL23">
+        <v>0.35</v>
       </c>
       <c r="AM23">
         <v>2.65</v>
@@ -2980,7 +3280,7 @@
         <v>39</v>
       </c>
       <c r="B24" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="C24">
         <v>3.5</v>
@@ -2992,7 +3292,7 @@
         <v>-111</v>
       </c>
       <c r="F24" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="G24">
         <v>822936</v>
@@ -3051,17 +3351,23 @@
       <c r="Y24">
         <v>1.0075</v>
       </c>
+      <c r="Z24">
+        <v>4</v>
+      </c>
       <c r="AA24" t="s">
         <v>44</v>
       </c>
+      <c r="AB24">
+        <v>0.06</v>
+      </c>
       <c r="AC24" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="AD24">
         <v>3.34</v>
       </c>
       <c r="AE24" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF24">
         <v>0.1603</v>
@@ -3071,6 +3377,18 @@
       </c>
       <c r="AH24">
         <v>0.22</v>
+      </c>
+      <c r="AI24">
+        <v>0.66</v>
+      </c>
+      <c r="AJ24">
+        <v>0.66</v>
+      </c>
+      <c r="AK24">
+        <v>0.44</v>
+      </c>
+      <c r="AL24">
+        <v>0.44</v>
       </c>
       <c r="AM24">
         <v>3.56</v>
@@ -3081,16 +3399,16 @@
         <v>39</v>
       </c>
       <c r="B25" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="F25" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="G25">
         <v>824874</v>
       </c>
       <c r="H25" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="I25">
         <v>3</v>
@@ -3144,16 +3462,16 @@
         <v>0.988</v>
       </c>
       <c r="AA25" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="AC25" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="AD25">
         <v>2.04</v>
       </c>
       <c r="AE25" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF25">
         <v>0.1484</v>
@@ -3173,7 +3491,7 @@
         <v>39</v>
       </c>
       <c r="B26" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="C26">
         <v>4.5</v>
@@ -3185,7 +3503,7 @@
         <v>-107</v>
       </c>
       <c r="F26" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="G26">
         <v>824874</v>
@@ -3244,17 +3562,23 @@
       <c r="Y26">
         <v>1.0258</v>
       </c>
+      <c r="Z26">
+        <v>6</v>
+      </c>
       <c r="AA26" t="s">
         <v>44</v>
       </c>
+      <c r="AB26">
+        <v>-0.19</v>
+      </c>
       <c r="AC26" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="AD26">
         <v>4.09</v>
       </c>
       <c r="AE26" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF26">
         <v>0.1743</v>
@@ -3264,6 +3588,18 @@
       </c>
       <c r="AH26">
         <v>0.22</v>
+      </c>
+      <c r="AI26">
+        <v>1.91</v>
+      </c>
+      <c r="AJ26">
+        <v>1.91</v>
+      </c>
+      <c r="AK26">
+        <v>1.69</v>
+      </c>
+      <c r="AL26">
+        <v>1.69</v>
       </c>
       <c r="AM26">
         <v>4.31</v>
@@ -3274,7 +3610,7 @@
         <v>39</v>
       </c>
       <c r="B27" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="C27">
         <v>4.5</v>
@@ -3286,7 +3622,7 @@
         <v>-170</v>
       </c>
       <c r="F27" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="G27">
         <v>823741</v>
@@ -3345,17 +3681,23 @@
       <c r="Y27">
         <v>1.0476</v>
       </c>
+      <c r="Z27">
+        <v>8</v>
+      </c>
       <c r="AA27" t="s">
         <v>44</v>
       </c>
+      <c r="AB27">
+        <v>0.39</v>
+      </c>
       <c r="AC27" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="AD27">
         <v>4.67</v>
       </c>
       <c r="AE27" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF27">
         <v>0.2087</v>
@@ -3365,6 +3707,18 @@
       </c>
       <c r="AH27">
         <v>0.22</v>
+      </c>
+      <c r="AI27">
+        <v>3.33</v>
+      </c>
+      <c r="AJ27">
+        <v>3.33</v>
+      </c>
+      <c r="AK27">
+        <v>3.11</v>
+      </c>
+      <c r="AL27">
+        <v>3.11</v>
       </c>
       <c r="AM27">
         <v>4.89</v>
@@ -3375,7 +3729,7 @@
         <v>39</v>
       </c>
       <c r="B28" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="C28">
         <v>5.5</v>
@@ -3387,7 +3741,7 @@
         <v>-113</v>
       </c>
       <c r="F28" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="G28">
         <v>823741</v>
@@ -3446,17 +3800,23 @@
       <c r="Y28">
         <v>1.0739</v>
       </c>
+      <c r="Z28">
+        <v>6</v>
+      </c>
       <c r="AA28" t="s">
         <v>44</v>
       </c>
+      <c r="AB28">
+        <v>0.51</v>
+      </c>
       <c r="AC28" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="AD28">
         <v>5.79</v>
       </c>
       <c r="AE28" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF28">
         <v>0.2356</v>
@@ -3466,6 +3826,18 @@
       </c>
       <c r="AH28">
         <v>0.22</v>
+      </c>
+      <c r="AI28">
+        <v>0.21</v>
+      </c>
+      <c r="AJ28">
+        <v>0.21</v>
+      </c>
+      <c r="AK28">
+        <v>-0.01</v>
+      </c>
+      <c r="AL28">
+        <v>0.01</v>
       </c>
       <c r="AM28">
         <v>6.01</v>
@@ -3476,10 +3848,10 @@
         <v>39</v>
       </c>
       <c r="B29" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="F29" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="G29">
         <v>824961</v>
@@ -3539,16 +3911,16 @@
         <v>1.0603</v>
       </c>
       <c r="AA29" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="AC29" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="AD29">
         <v>5.44</v>
       </c>
       <c r="AE29" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF29">
         <v>0.219</v>
@@ -3568,10 +3940,10 @@
         <v>39</v>
       </c>
       <c r="B30" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="F30" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="G30">
         <v>824961</v>
@@ -3631,16 +4003,16 @@
         <v>1.0306</v>
       </c>
       <c r="AA30" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="AC30" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="AD30">
         <v>6.09</v>
       </c>
       <c r="AE30" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="AF30">
         <v>0.2327</v>
@@ -3660,7 +4032,7 @@
         <v>39</v>
       </c>
       <c r="B31" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="C31">
         <v>7.5</v>
@@ -3672,7 +4044,7 @@
         <v>115</v>
       </c>
       <c r="F31" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="G31">
         <v>823986</v>
@@ -3731,17 +4103,23 @@
       <c r="Y31">
         <v>1.12</v>
       </c>
+      <c r="Z31">
+        <v>8</v>
+      </c>
       <c r="AA31" t="s">
         <v>44</v>
       </c>
+      <c r="AB31">
+        <v>3.4</v>
+      </c>
       <c r="AC31" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD31">
         <v>10.9</v>
       </c>
       <c r="AE31" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="AF31">
         <v>0.2859</v>
@@ -3751,6 +4129,18 @@
       </c>
       <c r="AH31">
         <v>0</v>
+      </c>
+      <c r="AI31">
+        <v>-2.9</v>
+      </c>
+      <c r="AJ31">
+        <v>2.9</v>
+      </c>
+      <c r="AK31">
+        <v>-2.9</v>
+      </c>
+      <c r="AL31">
+        <v>2.9</v>
       </c>
       <c r="AM31">
         <v>10.9</v>
@@ -3761,7 +4151,7 @@
         <v>39</v>
       </c>
       <c r="B32" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="C32">
         <v>3.5</v>
@@ -3773,7 +4163,7 @@
         <v>-130</v>
       </c>
       <c r="F32" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="G32">
         <v>823986</v>
@@ -3832,17 +4222,23 @@
       <c r="Y32">
         <v>0.9957</v>
       </c>
+      <c r="Z32">
+        <v>2</v>
+      </c>
       <c r="AA32" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB32">
+        <v>-0.96</v>
       </c>
       <c r="AC32" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD32">
         <v>2.32</v>
       </c>
       <c r="AE32" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF32">
         <v>0.1631</v>
@@ -3852,6 +4248,18 @@
       </c>
       <c r="AH32">
         <v>0.22</v>
+      </c>
+      <c r="AI32">
+        <v>-0.32</v>
+      </c>
+      <c r="AJ32">
+        <v>0.32</v>
+      </c>
+      <c r="AK32">
+        <v>-0.54</v>
+      </c>
+      <c r="AL32">
+        <v>0.54</v>
       </c>
       <c r="AM32">
         <v>2.54</v>
@@ -3862,7 +4270,7 @@
         <v>39</v>
       </c>
       <c r="B33" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="C33">
         <v>3.5</v>
@@ -3874,31 +4282,31 @@
         <v>-155</v>
       </c>
       <c r="F33" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="G33" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="H33" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="L33">
         <v>6</v>
       </c>
       <c r="S33" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="V33" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="AA33" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="AC33" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="AE33" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
     </row>
     <row r="34" spans="1:39" x14ac:dyDescent="0.25">
@@ -3906,10 +4314,10 @@
         <v>39</v>
       </c>
       <c r="B34" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="F34" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="G34">
         <v>824874</v>
@@ -3948,7 +4356,7 @@
         <v>0.39</v>
       </c>
       <c r="S34" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="T34">
         <v>0.225</v>
@@ -3969,16 +4377,16 @@
         <v>0.9749</v>
       </c>
       <c r="AA34" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="AC34" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="AD34">
         <v>3.21</v>
       </c>
       <c r="AE34" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF34">
         <v>0.1467</v>

</xml_diff>